<commit_message>
Tracker update: items.json, items.csv, Excel export
</commit_message>
<xml_diff>
--- a/data/ai-access-observatory.xlsx
+++ b/data/ai-access-observatory.xlsx
@@ -2739,7 +2739,7 @@
       </c>
       <c r="E89" s="7" t="inlineStr">
         <is>
-          <t>http://arxiv.org/abs/2608.18655v1</t>
+          <t>https://arxiv.org/abs/2608.18655v1</t>
         </is>
       </c>
     </row>
@@ -9210,7 +9210,7 @@
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>http://arxiv.org/abs/2608.18655v1</t>
+          <t>https://arxiv.org/abs/2608.18655v1</t>
         </is>
       </c>
     </row>

</xml_diff>